<commit_message>
Feature: new testcase: register user without input first name
</commit_message>
<xml_diff>
--- a/testcases/automation_practice_testcases.xlsx
+++ b/testcases/automation_practice_testcases.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="187">
   <si>
     <t xml:space="preserve">TEST CASE PLANNING AND EXECUTION TEMPLATE</t>
   </si>
@@ -278,6 +278,9 @@
   </si>
   <si>
     <t xml:space="preserve">User shouldn't able to register without input first name. Error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User can’t register. Error message: First name is required.</t>
   </si>
   <si>
     <t xml:space="preserve">001-13</t>
@@ -1966,8 +1969,12 @@
       <c r="E22" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F22" s="32"/>
-      <c r="G22" s="33"/>
+      <c r="F22" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="G22" s="33" t="s">
+        <v>35</v>
+      </c>
       <c r="H22" s="32"/>
       <c r="I22" s="32"/>
       <c r="J22" s="32"/>
@@ -1975,14 +1982,14 @@
     <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18"/>
       <c r="B23" s="30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="32" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F23" s="32"/>
       <c r="G23" s="33"/>
@@ -1992,14 +1999,14 @@
     </row>
     <row r="24" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F24" s="32"/>
       <c r="G24" s="33"/>
@@ -2009,14 +2016,14 @@
     </row>
     <row r="25" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="30" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="33"/>
@@ -2026,14 +2033,14 @@
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="30" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="33"/>
@@ -10975,13 +10982,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>29</v>
@@ -11017,7 +11024,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -11065,11 +11072,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -11121,19 +11128,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -11141,19 +11148,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -11161,19 +11168,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -11181,19 +11188,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -11201,19 +11208,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -11221,19 +11228,19 @@
     <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>
@@ -11241,19 +11248,19 @@
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="29"/>
       <c r="B17" s="30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F17" s="34"/>
       <c r="G17" s="33"/>
       <c r="H17" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I17" s="32"/>
       <c r="J17" s="32"/>
@@ -11261,19 +11268,19 @@
     <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="29"/>
       <c r="B18" s="30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F18" s="34"/>
       <c r="G18" s="33"/>
       <c r="H18" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I18" s="32"/>
       <c r="J18" s="32"/>
@@ -11281,19 +11288,19 @@
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18"/>
       <c r="B19" s="30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F19" s="34"/>
       <c r="G19" s="33"/>
       <c r="H19" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I19" s="32"/>
       <c r="J19" s="32"/>
@@ -11301,19 +11308,19 @@
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18"/>
       <c r="B20" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="32" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F20" s="34"/>
       <c r="G20" s="33"/>
       <c r="H20" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I20" s="32"/>
       <c r="J20" s="32"/>
@@ -11321,19 +11328,19 @@
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18"/>
       <c r="B21" s="30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="32" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F21" s="34"/>
       <c r="G21" s="33"/>
       <c r="H21" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I21" s="32"/>
       <c r="J21" s="32"/>
@@ -11341,19 +11348,19 @@
     <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18"/>
       <c r="B22" s="30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F22" s="34"/>
       <c r="G22" s="33"/>
       <c r="H22" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I22" s="32"/>
       <c r="J22" s="32"/>
@@ -11361,19 +11368,19 @@
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18"/>
       <c r="B23" s="30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F23" s="34"/>
       <c r="G23" s="33"/>
       <c r="H23" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
@@ -11381,19 +11388,19 @@
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18"/>
       <c r="B24" s="30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F24" s="34"/>
       <c r="G24" s="33"/>
       <c r="H24" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -11401,14 +11408,14 @@
     <row r="25" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18"/>
       <c r="B25" s="30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F25" s="34"/>
       <c r="G25" s="33"/>
@@ -11419,19 +11426,19 @@
     <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18"/>
       <c r="B26" s="30" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F26" s="34"/>
       <c r="G26" s="33"/>
       <c r="H26" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I26" s="32"/>
       <c r="J26" s="32"/>
@@ -11439,19 +11446,19 @@
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18"/>
       <c r="B27" s="30" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F27" s="34"/>
       <c r="G27" s="33"/>
       <c r="H27" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I27" s="32"/>
       <c r="J27" s="32"/>
@@ -11459,19 +11466,19 @@
     <row r="28" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18"/>
       <c r="B28" s="30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C28" s="31" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F28" s="34"/>
       <c r="G28" s="33"/>
       <c r="H28" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I28" s="32"/>
       <c r="J28" s="32"/>
@@ -11479,19 +11486,19 @@
     <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18"/>
       <c r="B29" s="30" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F29" s="34"/>
       <c r="G29" s="33"/>
       <c r="H29" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I29" s="32"/>
       <c r="J29" s="32"/>
@@ -11499,19 +11506,19 @@
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18"/>
       <c r="B30" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F30" s="34"/>
       <c r="G30" s="33"/>
       <c r="H30" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I30" s="32"/>
       <c r="J30" s="32"/>
@@ -11519,19 +11526,19 @@
     <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18"/>
       <c r="B31" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F31" s="34"/>
       <c r="G31" s="33"/>
       <c r="H31" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I31" s="32"/>
       <c r="J31" s="32"/>
@@ -11539,19 +11546,19 @@
     <row r="32" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18"/>
       <c r="B32" s="30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F32" s="34"/>
       <c r="G32" s="33"/>
       <c r="H32" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I32" s="32"/>
       <c r="J32" s="32"/>
@@ -11559,19 +11566,19 @@
     <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18"/>
       <c r="B33" s="30" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F33" s="34"/>
       <c r="G33" s="33"/>
       <c r="H33" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I33" s="32"/>
       <c r="J33" s="32"/>
@@ -11579,19 +11586,19 @@
     <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18"/>
       <c r="B34" s="30" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F34" s="34"/>
       <c r="G34" s="33"/>
       <c r="H34" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I34" s="32"/>
       <c r="J34" s="32"/>
@@ -11599,19 +11606,19 @@
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18"/>
       <c r="B35" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="32" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F35" s="34"/>
       <c r="G35" s="33"/>
       <c r="H35" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I35" s="32"/>
       <c r="J35" s="32"/>
@@ -11619,19 +11626,19 @@
     <row r="36" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18"/>
       <c r="B36" s="30" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="32" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F36" s="34"/>
       <c r="G36" s="33"/>
       <c r="H36" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I36" s="32"/>
       <c r="J36" s="32"/>
@@ -11639,19 +11646,19 @@
     <row r="37" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="18"/>
       <c r="B37" s="30" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F37" s="34"/>
       <c r="G37" s="33"/>
       <c r="H37" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I37" s="32"/>
       <c r="J37" s="32"/>
@@ -11659,14 +11666,14 @@
     <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18"/>
       <c r="B38" s="30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="32" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F38" s="34"/>
       <c r="G38" s="33"/>
@@ -20483,13 +20490,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>6</v>
@@ -20525,7 +20532,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -20573,11 +20580,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -20629,19 +20636,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -20649,19 +20656,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -20669,19 +20676,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -20689,19 +20696,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -20709,19 +20716,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -20729,19 +20736,19 @@
     <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>

</xml_diff>

<commit_message>
Feature: new testcase: register user without input first name (#217)
</commit_message>
<xml_diff>
--- a/testcases/automation_practice_testcases.xlsx
+++ b/testcases/automation_practice_testcases.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="187">
   <si>
     <t xml:space="preserve">TEST CASE PLANNING AND EXECUTION TEMPLATE</t>
   </si>
@@ -278,6 +278,9 @@
   </si>
   <si>
     <t xml:space="preserve">User shouldn't able to register without input first name. Error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User can’t register. Error message: First name is required.</t>
   </si>
   <si>
     <t xml:space="preserve">001-13</t>
@@ -1966,8 +1969,12 @@
       <c r="E22" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F22" s="32"/>
-      <c r="G22" s="33"/>
+      <c r="F22" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="G22" s="33" t="s">
+        <v>35</v>
+      </c>
       <c r="H22" s="32"/>
       <c r="I22" s="32"/>
       <c r="J22" s="32"/>
@@ -1975,14 +1982,14 @@
     <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18"/>
       <c r="B23" s="30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="32" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F23" s="32"/>
       <c r="G23" s="33"/>
@@ -1992,14 +1999,14 @@
     </row>
     <row r="24" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="30" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F24" s="32"/>
       <c r="G24" s="33"/>
@@ -2009,14 +2016,14 @@
     </row>
     <row r="25" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="30" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="33"/>
@@ -2026,14 +2033,14 @@
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="30" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="33"/>
@@ -10975,13 +10982,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>29</v>
@@ -11017,7 +11024,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -11065,11 +11072,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -11121,19 +11128,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -11141,19 +11148,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -11161,19 +11168,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -11181,19 +11188,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -11201,19 +11208,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -11221,19 +11228,19 @@
     <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>
@@ -11241,19 +11248,19 @@
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="29"/>
       <c r="B17" s="30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F17" s="34"/>
       <c r="G17" s="33"/>
       <c r="H17" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I17" s="32"/>
       <c r="J17" s="32"/>
@@ -11261,19 +11268,19 @@
     <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="29"/>
       <c r="B18" s="30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F18" s="34"/>
       <c r="G18" s="33"/>
       <c r="H18" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I18" s="32"/>
       <c r="J18" s="32"/>
@@ -11281,19 +11288,19 @@
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18"/>
       <c r="B19" s="30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F19" s="34"/>
       <c r="G19" s="33"/>
       <c r="H19" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I19" s="32"/>
       <c r="J19" s="32"/>
@@ -11301,19 +11308,19 @@
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18"/>
       <c r="B20" s="30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="32" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F20" s="34"/>
       <c r="G20" s="33"/>
       <c r="H20" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I20" s="32"/>
       <c r="J20" s="32"/>
@@ -11321,19 +11328,19 @@
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18"/>
       <c r="B21" s="30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="32" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F21" s="34"/>
       <c r="G21" s="33"/>
       <c r="H21" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I21" s="32"/>
       <c r="J21" s="32"/>
@@ -11341,19 +11348,19 @@
     <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18"/>
       <c r="B22" s="30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F22" s="34"/>
       <c r="G22" s="33"/>
       <c r="H22" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I22" s="32"/>
       <c r="J22" s="32"/>
@@ -11361,19 +11368,19 @@
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18"/>
       <c r="B23" s="30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F23" s="34"/>
       <c r="G23" s="33"/>
       <c r="H23" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
@@ -11381,19 +11388,19 @@
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18"/>
       <c r="B24" s="30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F24" s="34"/>
       <c r="G24" s="33"/>
       <c r="H24" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -11401,14 +11408,14 @@
     <row r="25" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18"/>
       <c r="B25" s="30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F25" s="34"/>
       <c r="G25" s="33"/>
@@ -11419,19 +11426,19 @@
     <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18"/>
       <c r="B26" s="30" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F26" s="34"/>
       <c r="G26" s="33"/>
       <c r="H26" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I26" s="32"/>
       <c r="J26" s="32"/>
@@ -11439,19 +11446,19 @@
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18"/>
       <c r="B27" s="30" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F27" s="34"/>
       <c r="G27" s="33"/>
       <c r="H27" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I27" s="32"/>
       <c r="J27" s="32"/>
@@ -11459,19 +11466,19 @@
     <row r="28" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18"/>
       <c r="B28" s="30" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C28" s="31" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F28" s="34"/>
       <c r="G28" s="33"/>
       <c r="H28" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I28" s="32"/>
       <c r="J28" s="32"/>
@@ -11479,19 +11486,19 @@
     <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18"/>
       <c r="B29" s="30" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F29" s="34"/>
       <c r="G29" s="33"/>
       <c r="H29" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I29" s="32"/>
       <c r="J29" s="32"/>
@@ -11499,19 +11506,19 @@
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18"/>
       <c r="B30" s="30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F30" s="34"/>
       <c r="G30" s="33"/>
       <c r="H30" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I30" s="32"/>
       <c r="J30" s="32"/>
@@ -11519,19 +11526,19 @@
     <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18"/>
       <c r="B31" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F31" s="34"/>
       <c r="G31" s="33"/>
       <c r="H31" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I31" s="32"/>
       <c r="J31" s="32"/>
@@ -11539,19 +11546,19 @@
     <row r="32" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18"/>
       <c r="B32" s="30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F32" s="34"/>
       <c r="G32" s="33"/>
       <c r="H32" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I32" s="32"/>
       <c r="J32" s="32"/>
@@ -11559,19 +11566,19 @@
     <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18"/>
       <c r="B33" s="30" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F33" s="34"/>
       <c r="G33" s="33"/>
       <c r="H33" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I33" s="32"/>
       <c r="J33" s="32"/>
@@ -11579,19 +11586,19 @@
     <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18"/>
       <c r="B34" s="30" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F34" s="34"/>
       <c r="G34" s="33"/>
       <c r="H34" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I34" s="32"/>
       <c r="J34" s="32"/>
@@ -11599,19 +11606,19 @@
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18"/>
       <c r="B35" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="32" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F35" s="34"/>
       <c r="G35" s="33"/>
       <c r="H35" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I35" s="32"/>
       <c r="J35" s="32"/>
@@ -11619,19 +11626,19 @@
     <row r="36" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18"/>
       <c r="B36" s="30" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="32" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F36" s="34"/>
       <c r="G36" s="33"/>
       <c r="H36" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I36" s="32"/>
       <c r="J36" s="32"/>
@@ -11639,19 +11646,19 @@
     <row r="37" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="18"/>
       <c r="B37" s="30" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F37" s="34"/>
       <c r="G37" s="33"/>
       <c r="H37" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I37" s="32"/>
       <c r="J37" s="32"/>
@@ -11659,14 +11666,14 @@
     <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18"/>
       <c r="B38" s="30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="32" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F38" s="34"/>
       <c r="G38" s="33"/>
@@ -20483,13 +20490,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>6</v>
@@ -20525,7 +20532,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -20573,11 +20580,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -20629,19 +20636,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -20649,19 +20656,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -20669,19 +20676,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -20689,19 +20696,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -20709,19 +20716,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -20729,19 +20736,19 @@
     <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>

</xml_diff>

<commit_message>
Feature: register user without input last name
</commit_message>
<xml_diff>
--- a/testcases/automation_practice_testcases.xlsx
+++ b/testcases/automation_practice_testcases.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="188">
   <si>
     <t xml:space="preserve">TEST CASE PLANNING AND EXECUTION TEMPLATE</t>
   </si>
@@ -290,6 +290,9 @@
   </si>
   <si>
     <t xml:space="preserve">User shouldn't able to register without input last name. Error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User can’t register. Error message: Last name is required.</t>
   </si>
   <si>
     <t xml:space="preserve">001-14</t>
@@ -1991,22 +1994,26 @@
       <c r="E23" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
+      <c r="F23" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>35</v>
+      </c>
       <c r="H23" s="32"/>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
     </row>
     <row r="24" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F24" s="32"/>
       <c r="G24" s="33"/>
@@ -2016,14 +2023,14 @@
     </row>
     <row r="25" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="33"/>
@@ -2033,14 +2040,14 @@
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="33"/>
@@ -10982,13 +10989,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>29</v>
@@ -11024,7 +11031,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -11072,11 +11079,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -11128,19 +11135,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -11148,19 +11155,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -11168,19 +11175,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -11188,19 +11195,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -11208,19 +11215,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -11228,19 +11235,19 @@
     <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>
@@ -11248,19 +11255,19 @@
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="29"/>
       <c r="B17" s="30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F17" s="34"/>
       <c r="G17" s="33"/>
       <c r="H17" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I17" s="32"/>
       <c r="J17" s="32"/>
@@ -11268,19 +11275,19 @@
     <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="29"/>
       <c r="B18" s="30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F18" s="34"/>
       <c r="G18" s="33"/>
       <c r="H18" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I18" s="32"/>
       <c r="J18" s="32"/>
@@ -11288,19 +11295,19 @@
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18"/>
       <c r="B19" s="30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="32" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" s="34"/>
       <c r="G19" s="33"/>
       <c r="H19" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I19" s="32"/>
       <c r="J19" s="32"/>
@@ -11308,19 +11315,19 @@
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18"/>
       <c r="B20" s="30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F20" s="34"/>
       <c r="G20" s="33"/>
       <c r="H20" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I20" s="32"/>
       <c r="J20" s="32"/>
@@ -11328,19 +11335,19 @@
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18"/>
       <c r="B21" s="30" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F21" s="34"/>
       <c r="G21" s="33"/>
       <c r="H21" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I21" s="32"/>
       <c r="J21" s="32"/>
@@ -11348,19 +11355,19 @@
     <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18"/>
       <c r="B22" s="30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F22" s="34"/>
       <c r="G22" s="33"/>
       <c r="H22" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I22" s="32"/>
       <c r="J22" s="32"/>
@@ -11368,19 +11375,19 @@
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18"/>
       <c r="B23" s="30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F23" s="34"/>
       <c r="G23" s="33"/>
       <c r="H23" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
@@ -11388,19 +11395,19 @@
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18"/>
       <c r="B24" s="30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F24" s="34"/>
       <c r="G24" s="33"/>
       <c r="H24" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -11408,14 +11415,14 @@
     <row r="25" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18"/>
       <c r="B25" s="30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F25" s="34"/>
       <c r="G25" s="33"/>
@@ -11426,19 +11433,19 @@
     <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18"/>
       <c r="B26" s="30" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F26" s="34"/>
       <c r="G26" s="33"/>
       <c r="H26" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I26" s="32"/>
       <c r="J26" s="32"/>
@@ -11446,19 +11453,19 @@
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18"/>
       <c r="B27" s="30" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F27" s="34"/>
       <c r="G27" s="33"/>
       <c r="H27" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I27" s="32"/>
       <c r="J27" s="32"/>
@@ -11466,19 +11473,19 @@
     <row r="28" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18"/>
       <c r="B28" s="30" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C28" s="31" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F28" s="34"/>
       <c r="G28" s="33"/>
       <c r="H28" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I28" s="32"/>
       <c r="J28" s="32"/>
@@ -11486,19 +11493,19 @@
     <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18"/>
       <c r="B29" s="30" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F29" s="34"/>
       <c r="G29" s="33"/>
       <c r="H29" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I29" s="32"/>
       <c r="J29" s="32"/>
@@ -11506,19 +11513,19 @@
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18"/>
       <c r="B30" s="30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F30" s="34"/>
       <c r="G30" s="33"/>
       <c r="H30" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I30" s="32"/>
       <c r="J30" s="32"/>
@@ -11526,19 +11533,19 @@
     <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18"/>
       <c r="B31" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F31" s="34"/>
       <c r="G31" s="33"/>
       <c r="H31" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I31" s="32"/>
       <c r="J31" s="32"/>
@@ -11546,19 +11553,19 @@
     <row r="32" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18"/>
       <c r="B32" s="30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F32" s="34"/>
       <c r="G32" s="33"/>
       <c r="H32" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I32" s="32"/>
       <c r="J32" s="32"/>
@@ -11566,19 +11573,19 @@
     <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18"/>
       <c r="B33" s="30" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F33" s="34"/>
       <c r="G33" s="33"/>
       <c r="H33" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I33" s="32"/>
       <c r="J33" s="32"/>
@@ -11586,19 +11593,19 @@
     <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18"/>
       <c r="B34" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F34" s="34"/>
       <c r="G34" s="33"/>
       <c r="H34" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I34" s="32"/>
       <c r="J34" s="32"/>
@@ -11606,19 +11613,19 @@
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18"/>
       <c r="B35" s="30" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="32" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F35" s="34"/>
       <c r="G35" s="33"/>
       <c r="H35" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I35" s="32"/>
       <c r="J35" s="32"/>
@@ -11626,19 +11633,19 @@
     <row r="36" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18"/>
       <c r="B36" s="30" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F36" s="34"/>
       <c r="G36" s="33"/>
       <c r="H36" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I36" s="32"/>
       <c r="J36" s="32"/>
@@ -11646,19 +11653,19 @@
     <row r="37" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="18"/>
       <c r="B37" s="30" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F37" s="34"/>
       <c r="G37" s="33"/>
       <c r="H37" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I37" s="32"/>
       <c r="J37" s="32"/>
@@ -11666,14 +11673,14 @@
     <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18"/>
       <c r="B38" s="30" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="32" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F38" s="34"/>
       <c r="G38" s="33"/>
@@ -20490,13 +20497,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>6</v>
@@ -20532,7 +20539,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -20580,11 +20587,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -20636,19 +20643,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -20656,19 +20663,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -20676,19 +20683,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -20696,19 +20703,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -20716,19 +20723,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -20736,19 +20743,19 @@
     <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>

</xml_diff>

<commit_message>
Feature: register user without input last name (#222)
</commit_message>
<xml_diff>
--- a/testcases/automation_practice_testcases.xlsx
+++ b/testcases/automation_practice_testcases.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="188">
   <si>
     <t xml:space="preserve">TEST CASE PLANNING AND EXECUTION TEMPLATE</t>
   </si>
@@ -290,6 +290,9 @@
   </si>
   <si>
     <t xml:space="preserve">User shouldn't able to register without input last name. Error message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User can’t register. Error message: Last name is required.</t>
   </si>
   <si>
     <t xml:space="preserve">001-14</t>
@@ -1991,22 +1994,26 @@
       <c r="E23" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
+      <c r="F23" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>35</v>
+      </c>
       <c r="H23" s="32"/>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
     </row>
     <row r="24" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F24" s="32"/>
       <c r="G24" s="33"/>
@@ -2016,14 +2023,14 @@
     </row>
     <row r="25" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F25" s="32"/>
       <c r="G25" s="33"/>
@@ -2033,14 +2040,14 @@
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="30" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F26" s="32"/>
       <c r="G26" s="33"/>
@@ -10982,13 +10989,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>29</v>
@@ -11024,7 +11031,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -11072,11 +11079,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -11128,19 +11135,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -11148,19 +11155,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -11168,19 +11175,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -11188,19 +11195,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -11208,19 +11215,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -11228,19 +11235,19 @@
     <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>
@@ -11248,19 +11255,19 @@
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="29"/>
       <c r="B17" s="30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F17" s="34"/>
       <c r="G17" s="33"/>
       <c r="H17" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I17" s="32"/>
       <c r="J17" s="32"/>
@@ -11268,19 +11275,19 @@
     <row r="18" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="29"/>
       <c r="B18" s="30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F18" s="34"/>
       <c r="G18" s="33"/>
       <c r="H18" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I18" s="32"/>
       <c r="J18" s="32"/>
@@ -11288,19 +11295,19 @@
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18"/>
       <c r="B19" s="30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="32" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" s="34"/>
       <c r="G19" s="33"/>
       <c r="H19" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I19" s="32"/>
       <c r="J19" s="32"/>
@@ -11308,19 +11315,19 @@
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="18"/>
       <c r="B20" s="30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F20" s="34"/>
       <c r="G20" s="33"/>
       <c r="H20" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I20" s="32"/>
       <c r="J20" s="32"/>
@@ -11328,19 +11335,19 @@
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18"/>
       <c r="B21" s="30" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F21" s="34"/>
       <c r="G21" s="33"/>
       <c r="H21" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I21" s="32"/>
       <c r="J21" s="32"/>
@@ -11348,19 +11355,19 @@
     <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18"/>
       <c r="B22" s="30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F22" s="34"/>
       <c r="G22" s="33"/>
       <c r="H22" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I22" s="32"/>
       <c r="J22" s="32"/>
@@ -11368,19 +11375,19 @@
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="18"/>
       <c r="B23" s="30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F23" s="34"/>
       <c r="G23" s="33"/>
       <c r="H23" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="32"/>
@@ -11388,19 +11395,19 @@
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="18"/>
       <c r="B24" s="30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F24" s="34"/>
       <c r="G24" s="33"/>
       <c r="H24" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
@@ -11408,14 +11415,14 @@
     <row r="25" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18"/>
       <c r="B25" s="30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F25" s="34"/>
       <c r="G25" s="33"/>
@@ -11426,19 +11433,19 @@
     <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18"/>
       <c r="B26" s="30" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D26" s="12"/>
       <c r="E26" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F26" s="34"/>
       <c r="G26" s="33"/>
       <c r="H26" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I26" s="32"/>
       <c r="J26" s="32"/>
@@ -11446,19 +11453,19 @@
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="18"/>
       <c r="B27" s="30" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D27" s="12"/>
       <c r="E27" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F27" s="34"/>
       <c r="G27" s="33"/>
       <c r="H27" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I27" s="32"/>
       <c r="J27" s="32"/>
@@ -11466,19 +11473,19 @@
     <row r="28" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="18"/>
       <c r="B28" s="30" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C28" s="31" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D28" s="12"/>
       <c r="E28" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F28" s="34"/>
       <c r="G28" s="33"/>
       <c r="H28" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I28" s="32"/>
       <c r="J28" s="32"/>
@@ -11486,19 +11493,19 @@
     <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="18"/>
       <c r="B29" s="30" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F29" s="34"/>
       <c r="G29" s="33"/>
       <c r="H29" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I29" s="32"/>
       <c r="J29" s="32"/>
@@ -11506,19 +11513,19 @@
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="18"/>
       <c r="B30" s="30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D30" s="12"/>
       <c r="E30" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F30" s="34"/>
       <c r="G30" s="33"/>
       <c r="H30" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I30" s="32"/>
       <c r="J30" s="32"/>
@@ -11526,19 +11533,19 @@
     <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="18"/>
       <c r="B31" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D31" s="12"/>
       <c r="E31" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F31" s="34"/>
       <c r="G31" s="33"/>
       <c r="H31" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I31" s="32"/>
       <c r="J31" s="32"/>
@@ -11546,19 +11553,19 @@
     <row r="32" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="18"/>
       <c r="B32" s="30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D32" s="12"/>
       <c r="E32" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F32" s="34"/>
       <c r="G32" s="33"/>
       <c r="H32" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I32" s="32"/>
       <c r="J32" s="32"/>
@@ -11566,19 +11573,19 @@
     <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="18"/>
       <c r="B33" s="30" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D33" s="12"/>
       <c r="E33" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F33" s="34"/>
       <c r="G33" s="33"/>
       <c r="H33" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I33" s="32"/>
       <c r="J33" s="32"/>
@@ -11586,19 +11593,19 @@
     <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18"/>
       <c r="B34" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D34" s="12"/>
       <c r="E34" s="32" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F34" s="34"/>
       <c r="G34" s="33"/>
       <c r="H34" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I34" s="32"/>
       <c r="J34" s="32"/>
@@ -11606,19 +11613,19 @@
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18"/>
       <c r="B35" s="30" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D35" s="12"/>
       <c r="E35" s="32" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F35" s="34"/>
       <c r="G35" s="33"/>
       <c r="H35" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I35" s="32"/>
       <c r="J35" s="32"/>
@@ -11626,19 +11633,19 @@
     <row r="36" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18"/>
       <c r="B36" s="30" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F36" s="34"/>
       <c r="G36" s="33"/>
       <c r="H36" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I36" s="32"/>
       <c r="J36" s="32"/>
@@ -11646,19 +11653,19 @@
     <row r="37" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="18"/>
       <c r="B37" s="30" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F37" s="34"/>
       <c r="G37" s="33"/>
       <c r="H37" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I37" s="32"/>
       <c r="J37" s="32"/>
@@ -11666,14 +11673,14 @@
     <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18"/>
       <c r="B38" s="30" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="32" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F38" s="34"/>
       <c r="G38" s="33"/>
@@ -20490,13 +20497,13 @@
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>6</v>
@@ -20532,7 +20539,7 @@
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
@@ -20580,11 +20587,11 @@
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="5"/>
@@ -20636,19 +20643,19 @@
     <row r="11" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="29"/>
       <c r="B11" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="33"/>
       <c r="H11" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I11" s="32"/>
       <c r="J11" s="32"/>
@@ -20656,19 +20663,19 @@
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29"/>
       <c r="B12" s="30" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="33"/>
       <c r="H12" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" s="32"/>
       <c r="J12" s="32"/>
@@ -20676,19 +20683,19 @@
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="32" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F13" s="35"/>
       <c r="G13" s="33"/>
       <c r="H13" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I13" s="32"/>
       <c r="J13" s="32"/>
@@ -20696,19 +20703,19 @@
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="32" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="33"/>
       <c r="H14" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="32"/>
@@ -20716,19 +20723,19 @@
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="30" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="32" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="33"/>
       <c r="H15" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I15" s="32"/>
       <c r="J15" s="32"/>
@@ -20736,19 +20743,19 @@
     <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="29"/>
       <c r="B16" s="30" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="33"/>
       <c r="H16" s="32" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I16" s="32"/>
       <c r="J16" s="32"/>

</xml_diff>